<commit_message>
feat: consult multiple records from spreadsheet
</commit_message>
<xml_diff>
--- a/data/entrada.xlsx
+++ b/data/entrada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,6 +501,40 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fernanda Rocha</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Registro Fantasma</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: compare expected and found status
</commit_message>
<xml_diff>
--- a/data/entrada.xlsx
+++ b/data/entrada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,7 +504,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>999</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -513,23 +513,6 @@
         </is>
       </c>
       <c r="C6" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Registro Fantasma</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>

</xml_diff>

<commit_message>
feat: add botcity web audit automation with evidences
</commit_message>
<xml_diff>
--- a/data/entrada.xlsx
+++ b/data/entrada.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,7 +480,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
     </row>
@@ -498,6 +498,23 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Registro Fantasma</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ativo</t>
         </is>
       </c>
     </row>

</xml_diff>